<commit_message>
session 20261021: IBA reset #2177 - control map, CLAUDE.md to pointers, history out of read path, memory cut, scoped rule delivery, SC15 close check, user guide rewrite (#2178-#2194)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -3435,7 +3435,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3498,6 +3498,8 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:D2"/>
@@ -6916,7 +6918,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7012,6 +7014,8 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:F2"/>
@@ -7510,7 +7514,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7573,6 +7577,8 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:D2"/>
@@ -7587,7 +7593,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT6"/>
+  <dimension ref="A1:AT8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8047,6 +8053,8 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
@@ -8061,7 +8069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8105,12 +8113,17 @@
       </c>
       <c r="E4" s="25" t="inlineStr">
         <is>
+          <t>-Mode</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
           <t>-Trace</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>switch (x to set)</t>
         </is>
@@ -8123,7 +8136,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" "&amp;D6&amp;" ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" "&amp;D6&amp;" ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -8208,7 +8221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8229,6 +8242,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -8299,6 +8313,8 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8310,7 +8326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8331,6 +8347,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -8391,6 +8408,8 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
session 20261021b: #2199/#2201 decisions applied -- templates, seed path, word-audit, narrative and word-registry-span stages, passage.suggest_boundary retired; backfill section registered; BUILD.md sec 370
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -8,56 +8,54 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Behaviour" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Book-Narrative" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build-Passages" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster-Assign" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster-Report" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config-Maintenance" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ContentIndex-Search" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ContentIndex-SizeProfile" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debate-Run" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalation" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export-Tables" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FolderPurpose" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lexicon-Parse" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spine-Check" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log-Retention" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest-Rebuild" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest-Search" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New-Word" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations-Ingest" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passage-Quality" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PathAudit" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prose" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw-Backfill" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registry-Report" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SchemaOverview-Report" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SchemaOverview-BibleRes" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpanAnalysis-Report" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start-Iba" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrongMeaning-Report" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrongVerse-Report" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VerseLexical" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WholeBookRead-Report" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WordRegistrySpan-Report" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue-Report" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue-Update" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BatchProgress" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharAnswer" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharReading" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClusterSubgroup" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VerseReading" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lexical-Readiness" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VerseMeta" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purge-SoftDeletes" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observation-Enhancer" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session-Close" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Narrative-Register" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy-NarrativeToLearning4Comfor" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelationalReading" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run-Stage1Batch" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build-Passages" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster-Assign" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster-Report" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config-Maintenance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ContentIndex-Search" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ContentIndex-SizeProfile" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debate-Run" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Escalation" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export-Tables" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FolderPurpose" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lexicon-Parse" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spine-Check" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log-Retention" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest-Rebuild" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest-Search" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New-Word" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations-Ingest" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Passage-Quality" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PathAudit" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prose" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw-Backfill" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registry-Report" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SchemaOverview-Report" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SchemaOverview-BibleRes" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpanAnalysis-Report" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start-Iba" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrongMeaning-Report" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StrongVerse-Report" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VerseLexical" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WholeBookRead-Report" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue-Report" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue-Update" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BatchProgress" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharAnswer" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharReading" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ClusterSubgroup" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VerseReading" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lexical-Readiness" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VerseMeta" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purge-SoftDeletes" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observation-Enhancer" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session-Close" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Narrative-Register" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy-NarrativeToLearning4Comfor" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelationalReading" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run-Stage1Batch" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -615,7 +613,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -676,12 +674,12 @@
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Book-Narrative.ps1</t>
+          <t>Build-Passages.ps1</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Run the book-narrative step for a book.</t>
+          <t>Build passage rows from a payload.</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -693,12 +691,12 @@
     <row r="7" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Build-Passages.ps1</t>
+          <t>Cluster-Assign.ps1</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Build passage rows from a payload.</t>
+          <t>Assign strongs to M-code clusters / validate assignment.</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
@@ -710,12 +708,12 @@
     <row r="8" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>Cluster-Assign.ps1</t>
+          <t>Cluster-Report.ps1</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Assign strongs to M-code clusters / validate assignment.</t>
+          <t>Cluster overview report.</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
@@ -727,12 +725,12 @@
     <row r="9" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>Cluster-Report.ps1</t>
+          <t>Config-Maintenance.ps1</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Cluster overview report.</t>
+          <t>THE sanctioned path for changing a cfg_* row.</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -744,12 +742,12 @@
     <row r="10" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>Config-Maintenance.ps1</t>
+          <t>ContentIndex-Search.ps1</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>THE sanctioned path for changing a cfg_* row.</t>
+          <t>Query the content search index.</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -761,12 +759,12 @@
     <row r="11" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>ContentIndex-Search.ps1</t>
+          <t>ContentIndex-SizeProfile.ps1</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Query the content search index.</t>
+          <t>Size-profile the content index.</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -778,46 +776,46 @@
     <row r="12" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>ContentIndex-SizeProfile.ps1</t>
+          <t>Debate-Run.ps1</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Size-profile the content index.</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>The debate pipeline (HIB/phenomenon/operation/closing) for a book.</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>n/a (not dispatcher-gated)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>Debate-Run.ps1</t>
+          <t>Escalation.ps1</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>The debate pipeline (HIB/phenomenon/operation/closing) for a book.</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>n/a (not dispatcher-gated)</t>
+          <t>See the researcher's own model sheet, 'escalation actions worksheet.xlsx' -- not rebuilt here, this tab is a pointer only.</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>Escalation.ps1</t>
+          <t>Export-Tables.ps1</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>See the researcher's own model sheet, 'escalation actions worksheet.xlsx' -- not rebuilt here, this tab is a pointer only.</t>
+          <t>Export one or more cfg_*/data tables to CSV.</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
@@ -829,12 +827,12 @@
     <row r="15" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>Export-Tables.ps1</t>
+          <t>FolderPurpose.ps1</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Export one or more cfg_*/data tables to CSV.</t>
+          <t>The folder_purpose governance mechanism (Methods A-D).</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -846,12 +844,12 @@
     <row r="16" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>FolderPurpose.ps1</t>
+          <t>Lexicon-Parse.ps1</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>The folder_purpose governance mechanism (Methods A-D).</t>
+          <t>Parse strong_lexicon / related-word data.</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
@@ -863,12 +861,12 @@
     <row r="17" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>Lexicon-Parse.ps1</t>
+          <t>Log-Retention.ps1</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Parse strong_lexicon / related-word data.</t>
+          <t>Apply log-retention rules (prune old logs).</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -880,12 +878,12 @@
     <row r="18" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t>Log-Retention.ps1</t>
+          <t>Manifest-Rebuild.ps1</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Apply log-retention rules (prune old logs).</t>
+          <t>Rebuild the file_manifest table.</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
@@ -897,12 +895,12 @@
     <row r="19" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t>Manifest-Rebuild.ps1</t>
+          <t>Manifest-Search.ps1</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>Rebuild the file_manifest table.</t>
+          <t>Search the file_manifest table.</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
@@ -914,12 +912,12 @@
     <row r="20" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A20" s="18" t="inlineStr">
         <is>
-          <t>Manifest-Search.ps1</t>
+          <t>New-Word.ps1</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>Search the file_manifest table.</t>
+          <t>Register a new word_registry entry and run its first-pass pipeline.</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
@@ -931,12 +929,12 @@
     <row r="21" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A21" s="18" t="inlineStr">
         <is>
-          <t>New-Word.ps1</t>
+          <t>Operations-Ingest.ps1</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>Register a new word_registry entry and run its first-pass pipeline.</t>
+          <t>Ingest a debate-step payload (hib/phenomenon/operation/closing).</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
@@ -948,12 +946,12 @@
     <row r="22" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t>Operations-Ingest.ps1</t>
+          <t>Passage-Quality.ps1</t>
         </is>
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Ingest a debate-step payload (hib/phenomenon/operation/closing).</t>
+          <t>Quality-check passages, optionally scoped to a book.</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
@@ -965,12 +963,12 @@
     <row r="23" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A23" s="18" t="inlineStr">
         <is>
-          <t>Passage-Quality.ps1</t>
+          <t>PathAudit.ps1</t>
         </is>
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>Quality-check passages, optionally scoped to a book.</t>
+          <t>Scan for hardcoded paths that should be config-driven.</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
@@ -982,12 +980,12 @@
     <row r="24" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>PathAudit.ps1</t>
+          <t>Prose.ps1</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>Scan for hardcoded paths that should be config-driven.</t>
+          <t>Prose store: extract/search/export/import/flag/status the programme prose.</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -999,12 +997,12 @@
     <row r="25" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A25" s="18" t="inlineStr">
         <is>
-          <t>Prose.ps1</t>
+          <t>Raw-Backfill.ps1</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>Prose store: extract/search/export/import/flag/status the programme prose.</t>
+          <t>Backfill span/strong_verse from raw span data for a book.</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
@@ -1016,12 +1014,12 @@
     <row r="26" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A26" s="18" t="inlineStr">
         <is>
-          <t>Raw-Backfill.ps1</t>
+          <t>Registry-Report.ps1</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>Backfill span/strong_verse from raw span data for a book.</t>
+          <t>word_registry overview report.</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
@@ -1033,12 +1031,12 @@
     <row r="27" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A27" s="18" t="inlineStr">
         <is>
-          <t>Registry-Report.ps1</t>
+          <t>Reports.ps1</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>word_registry overview report.</t>
+          <t>Word/book validation and report bundle.</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
@@ -1050,12 +1048,12 @@
     <row r="28" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Reports.ps1</t>
+          <t>SchemaOverview-Report.ps1</t>
         </is>
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>Word/book validation and report bundle.</t>
+          <t>Live iba.db schema overview report.</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -1065,34 +1063,34 @@
       </c>
     </row>
     <row r="29" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A29" s="18" t="inlineStr">
-        <is>
-          <t>SchemaOverview-Report.ps1</t>
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>SchemaOverview-BibleResearch-Report.ps1</t>
         </is>
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>Live iba.db schema overview report.</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
+          <t>Live bible_research.db schema overview report (merged against cfg_table/cfg_column, discrepancies flagged).</t>
+        </is>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>SchemaOverview-BibleResearch-Report.ps1</t>
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>SpanAnalysis-Report.ps1</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Live bible_research.db schema overview report (merged against cfg_table/cfg_column, discrepancies flagged).</t>
-        </is>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
+          <t>span table analysis report.</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1101,46 +1099,46 @@
     <row r="31" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A31" s="18" t="inlineStr">
         <is>
-          <t>SpanAnalysis-Report.ps1</t>
+          <t>Start-Iba.ps1</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>span table analysis report.</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Session bootstrap -- run once per session before any IBA work.</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>n/a (not dispatcher-gated)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A32" s="18" t="inlineStr">
         <is>
-          <t>Start-Iba.ps1</t>
+          <t>StrongMeaning-Report.ps1</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>Session bootstrap -- run once per session before any IBA work.</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>n/a (not dispatcher-gated)</t>
+          <t>strong_meaning_parsed/strong_lexicon coverage report.</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>StrongMeaning-Report.ps1</t>
+          <t>StrongVerse-Report.ps1</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>strong_meaning_parsed/strong_lexicon coverage report.</t>
+          <t>Report a word's strong&lt;-&gt;verse coverage.</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -1152,12 +1150,12 @@
     <row r="34" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>StrongVerse-Report.ps1</t>
+          <t>VerseLexical.ps1</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>Report a word's strong&lt;-&gt;verse coverage.</t>
+          <t>Run verse_lexical (L4b) derivation for a book/chapter range.</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
@@ -1169,12 +1167,12 @@
     <row r="35" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>VerseLexical.ps1</t>
+          <t>WholeBookRead-Report.ps1</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>Run verse_lexical (L4b) derivation for a book/chapter range.</t>
+          <t>Whole-book-read report for a book.</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
@@ -1184,51 +1182,51 @@
       </c>
     </row>
     <row r="36" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A36" s="18" t="inlineStr">
-        <is>
-          <t>WholeBookRead-Report.ps1</t>
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t>Catalogue-Report.ps1</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>Whole-book-read report for a book.</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="inlineStr">
+          <t>Structural review of wa_obs_question_catalogue (bible_research.db) -- no findings/joins. Read-only.</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A37" s="18" t="inlineStr">
-        <is>
-          <t>WordRegistrySpan-Report.ps1</t>
-        </is>
-      </c>
-      <c r="B37" s="19" t="inlineStr">
-        <is>
-          <t>Report a word's span coverage against its registry entry.</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Catalogue-Update.ps1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Validated partial UPDATE of one wa_obs_question_catalogue row by obs_id (source/last_modified/etc.). No history table.</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>Catalogue-Report.ps1</t>
-        </is>
-      </c>
-      <c r="B38" s="19" t="inlineStr">
-        <is>
-          <t>Structural review of wa_obs_question_catalogue (bible_research.db) -- no findings/joins. Read-only.</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Spine-Check.ps1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>The base-data spine check — verse/span/strong sync (FATAL per governance.base_data_spine, escalation #1613, researcher ruling 2026-09-10). Standalone, single-step work package, like Lexicon-Parse.ps1/Candidate-Quality.ps1. The strong-extended-meaning</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1237,12 +1235,12 @@
     <row r="39" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Catalogue-Update.ps1</t>
+          <t>BatchProgress.ps1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Validated partial UPDATE of one wa_obs_question_catalogue row by obs_id (source/last_modified/etc.). No history table.</t>
+          <t>Live progress monitor over run_batch -- resume/skip/crash-safeguard mechanism (#1756).</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1254,12 +1252,12 @@
     <row r="40" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Spine-Check.ps1</t>
+          <t>CharAnswer.ps1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>The base-data spine check — verse/span/strong sync (FATAL per governance.base_data_spine, escalation #1613, researcher ruling 2026-09-10). Standalone, single-step work package, like Lexicon-Parse.ps1/Candidate-Quality.ps1. The strong-extended-meaning</t>
+          <t>Stage 4 (char-answers) -- answer battery for one subgroup.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1271,12 +1269,12 @@
     <row r="41" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BatchProgress.ps1</t>
+          <t>CharReading.ps1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Live progress monitor over run_batch -- resume/skip/crash-safeguard mechanism (#1756).</t>
+          <t>Stage 3 (char-reading) -- corpus-wide subgroup reading.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1288,12 +1286,12 @@
     <row r="42" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CharAnswer.ps1</t>
+          <t>ClusterSubgroup.ps1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Stage 4 (char-answers) -- answer battery for one subgroup.</t>
+          <t>Stage 2 (char-subgroup) -- group cluster strongs into subgroups.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1305,12 +1303,12 @@
     <row r="43" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CharReading.ps1</t>
+          <t>Lexical-Readiness.ps1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Stage 3 (char-reading) -- corpus-wide subgroup reading.</t>
+          <t>Lexical readiness check.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1322,12 +1320,12 @@
     <row r="44" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ClusterSubgroup.ps1</t>
+          <t>VerseMeta.ps1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Stage 2 (char-subgroup) -- group cluster strongs into subgroups.</t>
+          <t>Verse-level metadata operations.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1339,12 +1337,12 @@
     <row r="45" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Lexical-Readiness.ps1</t>
+          <t>VerseReading.ps1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Lexical readiness check.</t>
+          <t>The `verse-reading` stage's WORD-LEVEL half (`lexical.meaning`, escalation #1706 Phase C pipeline stage 1; narrowed to word-level-only by the #1860 split, 2026-09-23) -- per-cluster, pre-subgroup Layer 2 pass answering M0.1 (Name and Naming) + M0.5 (</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1356,12 +1354,12 @@
     <row r="46" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A46" t="inlineStr">
         <is>
-          <t>VerseMeta.ps1</t>
+          <t>Purge-SoftDeletes.ps1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Verse-level metadata operations.</t>
+          <t>The soft-delete purge audit + execute + database retirement -- app-wide, both databases (escalation #1766/#1868/#1872/#1873). Standalone work package (chained=0 -- each action is an independent step you invoke separately, not a pipeline).</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1371,68 +1369,68 @@
       </c>
     </row>
     <row r="47" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>VerseReading.ps1</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>The `verse-reading` stage's WORD-LEVEL half (`lexical.meaning`, escalation #1706 Phase C pipeline stage 1; narrowed to word-level-only by the #1860 split, 2026-09-23) -- per-cluster, pre-subgroup Layer 2 pass answering M0.1 (Name and Naming) + M0.5 (</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>Observation-Enhancer.ps1</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>Apply a researcher-confirmed rule (selector+update) to ib_observation; logs every change (escalation #1778).</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Purge-SoftDeletes.ps1</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>The soft-delete purge audit + execute + database retirement -- app-wide, both databases (escalation #1766/#1868/#1872/#1873). Standalone work package (chained=0 -- each action is an independent step you invoke separately, not a pipeline).</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>Session-Close.ps1</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>Session-close detection (escalation #1875; rebuilt #2173, SC1-SC14): session and window, spine (FATAL first), researcher's words recorded, open items in the register, analysis integrity, rule compliance evidence, session log, decisions' targets, BUIL</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A49" s="23" t="inlineStr">
-        <is>
-          <t>Observation-Enhancer.ps1</t>
-        </is>
-      </c>
-      <c r="B49" s="23" t="inlineStr">
-        <is>
-          <t>Apply a researcher-confirmed rule (selector+update) to ib_observation; logs every change (escalation #1778).</t>
-        </is>
-      </c>
-      <c r="C49" s="23" t="inlineStr">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Narrative-Register.ps1</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>The narrative claim register in iba.db (escalation #2110): add and edit claims, link them to the passages that tell them, record a weave, search, show a claim's history, check against the chapter files, and publish the three register files. Every act</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A50" s="23" t="inlineStr">
-        <is>
-          <t>Session-Close.ps1</t>
-        </is>
-      </c>
-      <c r="B50" s="23" t="inlineStr">
-        <is>
-          <t>Session-close detection (escalation #1875; rebuilt #2173, SC1-SC14): session and window, spine (FATAL first), researcher's words recorded, open items in the register, analysis integrity, rule compliance evidence, session log, decisions' targets, BUIL</t>
-        </is>
-      </c>
-      <c r="C50" s="23" t="inlineStr">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Compliance.ps1</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>The session compliance file (escalation #2173 P2): the governance settings, behaviour rules and escalation rules, restated at start and proved at close.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1441,12 +1439,12 @@
     <row r="51" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Narrative-Register.ps1</t>
+          <t>Copy-NarrativeToLearning4Comfort.ps1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>The narrative claim register in iba.db (escalation #2110): add and edit claims, link them to the passages that tell them, record a weave, search, show a claim's history, check against the chapter files, and publish the three register files. Every act</t>
+          <t>Copy the current inner-being narrative files to the learning4comfort publication inbox (escalation #1941). This project never publishes to GitHub itself; the learning4comfort repo prepares, reviews and publishes from its inbox.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1458,12 +1456,12 @@
     <row r="52" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Compliance.ps1</t>
+          <t>RelationalReading.ps1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>The session compliance file (escalation #2173 P2): the governance settings, behaviour rules and escalation rules, restated at start and proved at close.</t>
+          <t>The `verse-reading` stage's RELATIONAL half (`lexical.relational`, escalation #1860 word-level/ relational split, 2026-09-23) -- per-cluster, pre-subgroup Layer 2 pass answering M0.6.5/M0.6.6/ D7.7.1/M0.7.1-16/M0.8.1. Standalone single-step entry poi</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1475,49 +1473,15 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Copy-NarrativeToLearning4Comfort.ps1</t>
+          <t>Run-Stage1Batch.ps1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Copy the current inner-being narrative files to the learning4comfort publication inbox (escalation #1941). This project never publishes to GitHub itself; the learning4comfort repo prepares, reviews and publishes from its inbox.</t>
+          <t xml:space="preserve">Batch controller for `lexical.meaning` (Stage 1 verse-reading) -- runs an explicit list of clusters sequentially, unattended, so a multi-cluster pass can run in the background while progress is watched separately with `BatchProgress.ps1` (escalation </t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>RelationalReading.ps1</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>The `verse-reading` stage's RELATIONAL half (`lexical.relational`, escalation #1860 word-level/ relational split, 2026-09-23) -- per-cluster, pre-subgroup Layer 2 pass answering M0.6.5/M0.6.6/ D7.7.1/M0.7.1-16/M0.8.1. Standalone single-step entry poi</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Run-Stage1Batch.ps1</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Batch controller for `lexical.meaning` (Stage 1 verse-reading) -- runs an explicit list of clusters sequentially, unattended, so a multi-cluster pass can run in the background while progress is watched separately with `BatchProgress.ps1` (escalation </t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1537,113 +1501,6 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Debate-Run.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>The debate pipeline (HIB/phenomenon/operation/closing) for a book.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>-Book</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-Chapters</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>-Range</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>-BookLabel</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>-Step</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>hib.set|passage.build|phenomenon.set|operation.set|closing.set</t>
-        </is>
-      </c>
-      <c r="H5" s="17" t="inlineStr">
-        <is>
-          <t>resume a specific run</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>iba\app\ps\Debate-Run.ps1</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" "&amp;G6&amp;" ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6&lt;&gt;"",$I$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:I2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1673,7 +1530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -1776,7 +1633,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -1898,7 +1755,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -1975,6 +1832,83 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Spine-Check.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The base-data spine check — verse/span/strong sync (FATAL per governance.base_data_spine, escalation #1613, researcher ruling 2026-09-10). Standalone, single-step work package, like Lexicon-Parse.ps1/Candidate-Quality.ps1. The strong-extended-meaning-parse completeness check + its discoverability pass were REMOVED 2026-09-11 (escalation #1681/#1684/#1686) — they checked coverage against strong_meaning_parsed/strong_lsj_parsed/strong_mounce_parsed, which were retired/frozen on 2026-09-10 and are no longer maintained. See handlers/spine.py module docstring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1"/>
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customHeight="1">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Spine-Check.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1995,56 +1929,50 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>Spine-Check.ps1</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Log-Retention.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>The base-data spine check — verse/span/strong sync (FATAL per governance.base_data_spine, escalation #1613, researcher ruling 2026-09-10). Standalone, single-step work package, like Lexicon-Parse.ps1/Candidate-Quality.ps1. The strong-extended-meaning-parse completeness check + its discoverability pass were REMOVED 2026-09-11 (escalation #1681/#1684/#1686) — they checked coverage against strong_meaning_parsed/strong_lsj_parsed/strong_mounce_parsed, which were retired/frozen on 2026-09-10 and are no longer maintained. See handlers/spine.py module docstring.</t>
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Apply log-retention rules (prune old logs).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18.75" customHeight="1"/>
     <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>script</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>compiled command (copy/paste)</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>-RunId</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>-Trace</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18.75" customHeight="1">
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-    </row>
+    <row r="5" ht="18.75" customHeight="1"/>
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>iba\app\ps\Spine-Check.ps1</t>
-        </is>
-      </c>
-      <c r="B6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Log-Retention.ps1</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
         <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
         <v/>
       </c>
@@ -2074,14 +2002,14 @@
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Log-Retention.ps1</t>
+          <t>Manifest-Rebuild.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Apply log-retention rules (prune old logs).</t>
+          <t>Rebuild the file_manifest table.</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2040,7 @@
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\Log-Retention.ps1</t>
+          <t>iba\app\ps\Manifest-Rebuild.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
@@ -2129,77 +2057,6 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Manifest-Rebuild.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Rebuild the file_manifest table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customHeight="1"/>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>iba\app\ps\Manifest-Rebuild.ps1</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -2281,7 +2138,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -2378,6 +2235,113 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Operations-Ingest.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Ingest a debate-step payload (hib/phenomenon/operation/closing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1"/>
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>-Step</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-Book</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>-Chapters</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>-Range</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>-PayloadPath</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>hib.set|phenomenon.set|operation.set|closing.set</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>path to the payload JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Operations-Ingest.ps1</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6&lt;&gt;"",$I$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2471,25 +2435,25 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="9"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Operations-Ingest.ps1</t>
+          <t>Passage-Quality.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Ingest a debate-step payload (hib/phenomenon/operation/closing).</t>
+          <t>Quality-check passages, optionally scoped to a book.</t>
         </is>
       </c>
     </row>
@@ -2507,35 +2471,15 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>-Step</t>
+          <t>-Book</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-Book</t>
+          <t>-RunId</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>-Chapters</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>-Range</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>-PayloadPath</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>-Trace</t>
         </is>
@@ -2544,29 +2488,24 @@
     <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>hib.set|phenomenon.set|operation.set|closing.set</t>
-        </is>
-      </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>path to the payload JSON</t>
+          <t>omit for all books</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\Operations-Ingest.ps1</t>
+          <t>iba\app\ps\Passage-Quality.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6&lt;&gt;"",$I$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2589,14 +2528,14 @@
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Passage-Quality.ps1</t>
+          <t>PathAudit.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Quality-check passages, optionally scoped to a book.</t>
+          <t>Scan for hardcoded paths that should be config-driven.</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2553,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>-Book</t>
+          <t>-Action</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -2631,18 +2570,18 @@
     <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>omit for all books</t>
+          <t>Scan</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\Passage-Quality.ps1</t>
+          <t>iba\app\ps\PathAudit.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -2655,88 +2594,6 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PathAudit.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Scan for hardcoded paths that should be config-driven.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>-Action</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>Scan</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>iba\app\ps\PathAudit.ps1</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -2968,7 +2825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -3055,7 +2912,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -3126,7 +2983,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -3208,6 +3065,77 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SchemaOverview-Report.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Live iba.db schema overview report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1"/>
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customHeight="1"/>
+    <row r="6" ht="66.75" customFormat="1" customHeight="1" s="18">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>iba\app\ps\SchemaOverview-Report.ps1</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3230,14 +3158,14 @@
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SchemaOverview-Report.ps1</t>
+          <t>SchemaOverview-BibleResearch-Report.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Live iba.db schema overview report.</t>
+          <t>Live bible_research.db schema overview report -- merged against cfg_table/cfg_column, table+column level, discrepancies flagged.</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3196,7 @@
     <row r="6" ht="66.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\SchemaOverview-Report.ps1</t>
+          <t>iba\app\ps\SchemaOverview-BibleResearch-Report.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
@@ -3301,14 +3229,14 @@
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SchemaOverview-BibleResearch-Report.ps1</t>
+          <t>SpanAnalysis-Report.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Live bible_research.db schema overview report -- merged against cfg_table/cfg_column, table+column level, discrepancies flagged.</t>
+          <t>span table analysis report.</t>
         </is>
       </c>
     </row>
@@ -3336,10 +3264,10 @@
       </c>
     </row>
     <row r="5" ht="18.75" customHeight="1"/>
-    <row r="6" ht="66.75" customFormat="1" customHeight="1" s="18">
+    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\SchemaOverview-BibleResearch-Report.ps1</t>
+          <t>iba\app\ps\SpanAnalysis-Report.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
@@ -3361,7 +3289,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3372,14 +3300,14 @@
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SpanAnalysis-Report.ps1</t>
+          <t>Start-Iba.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>span table analysis report.</t>
+          <t>Session bootstrap -- run once per session before any IBA work.</t>
         </is>
       </c>
     </row>
@@ -3397,24 +3325,25 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customHeight="1"/>
+          <t>-Reset</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>full reset</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\SpanAnalysis-Report.ps1</t>
+          <t>iba\app\ps\Start-Iba.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6&lt;&gt;"",$C$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -3432,25 +3361,27 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="6"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="7"/>
+    <col width="11.4" customWidth="1" min="8" max="8"/>
+    <col width="11.4" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Book-Narrative.ps1</t>
+          <t>Build-Passages.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Run the book-narrative step for a book.</t>
+          <t>Build passage rows from a payload.</t>
         </is>
       </c>
     </row>
@@ -3473,35 +3404,46 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-BookLabel</t>
+          <t>-Chapters</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>-RunId</t>
+          <t>-Range</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
+          <t>-PayloadPath</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
           <t>-Trace</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18.75" customHeight="1"/>
+    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>path to the payload JSON</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\Book-Narrative.ps1</t>
+          <t>iba\app\ps\Build-Passages.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3524,14 +3466,14 @@
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Start-Iba.ps1</t>
+          <t>StrongMeaning-Report.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Session bootstrap -- run once per session before any IBA work.</t>
+          <t>strong_meaning_parsed/strong_lexicon coverage report.</t>
         </is>
       </c>
     </row>
@@ -3549,35 +3491,24 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>-Reload</t>
+          <t>-RunId</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-Reset</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>reseed config from source</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="inlineStr">
-        <is>
-          <t>full reset</t>
-        </is>
-      </c>
-    </row>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customHeight="1"/>
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\Start-Iba.ps1</t>
+          <t>iba\app\ps\StrongMeaning-Report.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6&lt;&gt;"",$C$4&amp;" ","")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -3590,77 +3521,6 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>StrongMeaning-Report.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>strong_meaning_parsed/strong_lexicon coverage report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customHeight="1"/>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>iba\app\ps\StrongMeaning-Report.ps1</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -3747,7 +3607,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -4210,7 +4070,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -4291,83 +4151,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>WordRegistrySpan-Report.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Report a word's span coverage against its registry entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>-Word</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customHeight="1"/>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>iba\app\ps\WordRegistrySpan-Report.ps1</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4433,7 +4217,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -4541,7 +4325,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -4632,7 +4416,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -4724,121 +4508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="7"/>
-    <col width="11.4" customWidth="1" min="8" max="8"/>
-    <col width="11.4" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Build-Passages.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Build passage rows from a payload.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>-Book</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-Chapters</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>-Range</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>-PayloadPath</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-      <c r="H4" s="22" t="inlineStr">
-        <is>
-          <t>-Suggest</t>
-        </is>
-      </c>
-      <c r="I4" s="22" t="inlineStr">
-        <is>
-          <t>-Confirm</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="F5" s="17" t="inlineStr">
-        <is>
-          <t>path to the payload JSON</t>
-        </is>
-      </c>
-      <c r="H5" s="23" t="inlineStr">
-        <is>
-          <t>switch -- propose the next candidate passage boundary from cheap mechanical proxy signals (no table write, pauses for confirm/adjust); mutually exclusive with -Chapters/-Range</t>
-        </is>
-      </c>
-      <c r="I5" s="23" t="inlineStr">
-        <is>
-          <t>switch -- only with -Suggest: accept the suggestion verbatim, straight into passage.build (still needs -PayloadPath)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>iba\app\ps\Build-Passages.ps1</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")&amp;IF(I6&lt;&gt;"",$I$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:G2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -4919,6 +4589,284 @@
       </c>
       <c r="B6" s="5">
         <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="6"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ClusterSubgroup.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Stage 2 (char-subgroup) -- group a cluster's member strongs into meaning-based subgroups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1"/>
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>-ClusterCode</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>-Live</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="D5" s="17" t="n"/>
+    </row>
+    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>iba\app\ps\ClusterSubgroup.ps1</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cluster-Assign.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Assign strongs to M-code clusters / validate assignment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1"/>
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>-Step</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Assign|Validate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Cluster-Assign.ps1</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="6"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>VerseReading.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The `verse-reading` stage's WORD-LEVEL half (`lexical.meaning`, escalation #1706 Phase C pipeline stage 1; narrowed to word-level-only by the #1860 split, 2026-09-23) -- per-cluster, pre-subgroup Layer 2 pass answering M0.1 (Name and Naming) + M0.5 (Lexical and Semantic Analysis) only. Standalone single-step entry point onto the `verse-lexical` work package's `lexical.meaning` step (ordinal 6) -- this step didn't have a PS entry point until now, found live building this (`cfg_behaviour_rule` `every-interactive-module-needs-ps-script`). Run `RelationalReading.ps1` (`lexical.relational`) next for the same cluster once this has covered its verses -- the relational family (M0.6.5/M0.6.6/D7.7.1/M0.7/M0.8.1) moved there, with a readiness gate requiring this step's own output first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1"/>
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>-ClusterCode</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>-VerseList</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>-Live</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>-Force</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\VerseReading.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -4942,22 +4890,19 @@
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="22" bestFit="1" customWidth="1" min="3" max="6"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ClusterSubgroup.ps1</t>
+          <t>Lexical-Readiness.ps1</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Stage 2 (char-subgroup) -- group a cluster's member strongs into meaning-based subgroups.</t>
+          <t>Lexical readiness check (lexical.readiness).</t>
         </is>
       </c>
     </row>
@@ -4975,24 +4920,12 @@
       </c>
       <c r="C4" s="22" t="inlineStr">
         <is>
-          <t>-ClusterCode</t>
-        </is>
-      </c>
-      <c r="D4" s="22" t="inlineStr">
-        <is>
-          <t>-Live</t>
-        </is>
-      </c>
-      <c r="E4" s="22" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="F4" s="22" t="inlineStr">
-        <is>
           <t>-Trace</t>
         </is>
       </c>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="D5" s="17" t="n"/>
@@ -5000,11 +4933,11 @@
     <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>iba\app\ps\ClusterSubgroup.ps1</t>
+          <t>iba\app\ps\Lexical-Readiness.ps1</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6&lt;&gt;"",$C$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -5017,187 +4950,6 @@
 </file>
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="6"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>VerseReading.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>The `verse-reading` stage's WORD-LEVEL half (`lexical.meaning`, escalation #1706 Phase C pipeline stage 1; narrowed to word-level-only by the #1860 split, 2026-09-23) -- per-cluster, pre-subgroup Layer 2 pass answering M0.1 (Name and Naming) + M0.5 (Lexical and Semantic Analysis) only. Standalone single-step entry point onto the `verse-lexical` work package's `lexical.meaning` step (ordinal 6) -- this step didn't have a PS entry point until now, found live building this (`cfg_behaviour_rule` `every-interactive-module-needs-ps-script`). Run `RelationalReading.ps1` (`lexical.relational`) next for the same cluster once this has covered its verses -- the relational family (M0.6.5/M0.6.6/D7.7.1/M0.7/M0.8.1) moved there, with a readiness gate requiring this step's own output first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="25" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="25" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>-ClusterCode</t>
-        </is>
-      </c>
-      <c r="D4" s="25" t="inlineStr">
-        <is>
-          <t>-VerseList</t>
-        </is>
-      </c>
-      <c r="E4" s="25" t="inlineStr">
-        <is>
-          <t>-Live</t>
-        </is>
-      </c>
-      <c r="F4" s="25" t="inlineStr">
-        <is>
-          <t>-Force</t>
-        </is>
-      </c>
-      <c r="G4" s="25" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="H4" s="25" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>iba\app\ps\VerseReading.ps1</t>
-        </is>
-      </c>
-      <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Lexical-Readiness.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Lexical readiness check (lexical.readiness).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="22" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-    </row>
-    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="D5" s="17" t="n"/>
-    </row>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>iba\app\ps\Lexical-Readiness.ps1</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6&lt;&gt;"",$C$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -5283,7 +5035,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -5380,7 +5132,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5486,7 +5238,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -5563,7 +5315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -6037,7 +5789,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6119,89 +5871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="22" bestFit="1" customWidth="1" min="3" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Cluster-Assign.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>Assign strongs to M-code clusters / validate assignment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18.75" customHeight="1"/>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>-Step</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>Assign|Validate</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>iba\app\ps\Cluster-Assign.ps1</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6268,7 +5938,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6370,99 +6040,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>Run-Stage1Batch.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Batch controller for `lexical.meaning` (Stage 1 verse-reading) -- runs an explicit list of clusters sequentially, unattended, so a multi-cluster pass can run in the background while progress is watched separately with `BatchProgress.ps1` (escalation #1756's own monitor, read- only over `run_batch` -- `lexical.meaning` already writes there via `batchcontrol.py`, so no new monitoring mechanism was needed, only this orchestration layer).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="25" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="25" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>-ClusterCodes</t>
-        </is>
-      </c>
-      <c r="D4" s="25" t="inlineStr">
-        <is>
-          <t>-Live</t>
-        </is>
-      </c>
-      <c r="E4" s="25" t="inlineStr">
-        <is>
-          <t>-MaxTotalCostUsd</t>
-        </is>
-      </c>
-      <c r="F4" s="25" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="G4" s="25" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>iba\app\ps\Run-Stage1Batch.ps1</t>
-        </is>
-      </c>
-      <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -6533,7 +6111,99 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Run-Stage1Batch.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Batch controller for `lexical.meaning` (Stage 1 verse-reading) -- runs an explicit list of clusters sequentially, unattended, so a multi-cluster pass can run in the background while progress is watched separately with `BatchProgress.ps1` (escalation #1756's own monitor, read- only over `run_batch` -- `lexical.meaning` already writes there via `batchcontrol.py`, so no new monitoring mechanism was needed, only this orchestration layer).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>-ClusterCodes</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>-Live</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>-MaxTotalCostUsd</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Run-Stage1Batch.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -6682,7 +6352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -6769,7 +6439,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -6838,4 +6508,111 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="60" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22" bestFit="1" customWidth="1" min="3" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Debate-Run.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>The debate pipeline (HIB/phenomenon/operation/closing) for a book.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1"/>
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>-Book</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-Chapters</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>-Range</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>-BookLabel</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>-Step</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>hib.set|passage.build|phenomenon.set|operation.set|closing.set</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="inlineStr">
+        <is>
+          <t>resume a specific run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18.75" customFormat="1" customHeight="1" s="18">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Debate-Run.ps1</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" "&amp;G6&amp;" ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6&lt;&gt;"",$I$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
session 20261022: #2172 reading process built -- Strand-Reading.ps1 (define, context, record, gather, map, derive, rewrite, account), claims told per block, the narrative written in iba.db with chapters as exports, the strand close gate, governance.narrative_home; tests 84/84 on copies; catch-up plan B-D for decision; #2213 raised, #2214 #2215 fixed; BUILD.md sec 386-387
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -52,10 +52,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observation-Enhancer" sheetId="44" state="visible" r:id="rId44"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session-Close" sheetId="45" state="visible" r:id="rId45"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Narrative-Register" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy-NarrativeToLearning4Comfor" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelationalReading" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run-Stage1Batch" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strand-Reading" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy-NarrativeToLearning4Comfor" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelationalReading" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run-Stage1Batch" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -613,7 +614,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1410,7 +1411,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>The narrative claim register in iba.db (escalation #2110): add and edit claims, link them to the passages that tell them, record a weave, search, show a claim's history, check against the chapter files, and publish the three register files. Every act</t>
+          <t>The narrative claim register in iba.db (escalation #2110): add and edit claims, link them to the blocks that tell them, search, show a claim's history, check the chapters against the database, and publish the three register files. The narrative itself is written through Strand-Reading.ps1 -Step Rewrite (#2172). Every action dispatches through run.py, work package narrative-register.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1482,6 +1483,23 @@
         </is>
       </c>
       <c r="C53" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Strand-Reading.ps1</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>The reading process (escalation #2172): a strand defined, then context, record, gather, map, derive, rewrite and account. Every step dispatches through run.py, work package strand-reading; the JSON shapes are in lib/strandreading.py.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -3289,7 +3307,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5341,7 +5359,7 @@
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The narrative claim register in iba.db (escalation #2110): add and edit claims, link them to the passages that tell them, record a weave, search, show a claim's history, check against the chapter files, and publish the three register files. Every action dispatches through run.py, work package narrative-register.</t>
+          <t>The narrative claim register in iba.db (escalation #2110): add and edit claims, link them to the blocks that tell them, search, show a claim's history, check the chapters against the database, and publish the three register files. The narrative itself is written through Strand-Reading.ps1 -Step Rewrite (#2172). Every action dispatches through run.py, work package narrative-register.</t>
         </is>
       </c>
     </row>
@@ -5434,154 +5452,150 @@
       </c>
       <c r="R4" s="25" t="inlineStr">
         <is>
-          <t>-Passage</t>
+          <t>-Kind</t>
         </is>
       </c>
       <c r="S4" s="25" t="inlineStr">
         <is>
-          <t>-Kind</t>
+          <t>-Part</t>
         </is>
       </c>
       <c r="T4" s="25" t="inlineStr">
         <is>
-          <t>-Part</t>
+          <t>-Heading</t>
         </is>
       </c>
       <c r="U4" s="25" t="inlineStr">
         <is>
-          <t>-Heading</t>
+          <t>-NewHeading</t>
         </is>
       </c>
       <c r="V4" s="25" t="inlineStr">
         <is>
-          <t>-NewHeading</t>
+          <t>-Ordinal</t>
         </is>
       </c>
       <c r="W4" s="25" t="inlineStr">
         <is>
-          <t>-Ordinal</t>
+          <t>-Level</t>
         </is>
       </c>
       <c r="X4" s="25" t="inlineStr">
         <is>
-          <t>-Level</t>
+          <t>-LastVersion</t>
         </is>
       </c>
       <c r="Y4" s="25" t="inlineStr">
         <is>
-          <t>-LastVersion</t>
+          <t>-NewNumber</t>
         </is>
       </c>
       <c r="Z4" s="25" t="inlineStr">
         <is>
-          <t>-NewNumber</t>
+          <t>-Title</t>
         </is>
       </c>
       <c r="AA4" s="25" t="inlineStr">
         <is>
-          <t>-Title</t>
+          <t>-State</t>
         </is>
       </c>
       <c r="AB4" s="25" t="inlineStr">
         <is>
-          <t>-State</t>
+          <t>-CurrentFile</t>
         </is>
       </c>
       <c r="AC4" s="25" t="inlineStr">
         <is>
-          <t>-CurrentFile</t>
+          <t>-CurrentVersion</t>
         </is>
       </c>
       <c r="AD4" s="25" t="inlineStr">
         <is>
-          <t>-CurrentVersion</t>
+          <t>-ReadingOrder</t>
         </is>
       </c>
       <c r="AE4" s="25" t="inlineStr">
         <is>
-          <t>-ReadingOrder</t>
+          <t>-Inactive</t>
         </is>
       </c>
       <c r="AF4" s="25" t="inlineStr">
         <is>
-          <t>-Inactive</t>
+          <t>-Purpose</t>
         </is>
       </c>
       <c r="AG4" s="25" t="inlineStr">
         <is>
-          <t>-Purpose</t>
+          <t>-PurposeRef</t>
         </is>
       </c>
       <c r="AH4" s="25" t="inlineStr">
         <is>
-          <t>-PurposeRef</t>
+          <t>-After</t>
         </is>
       </c>
       <c r="AI4" s="25" t="inlineStr">
         <is>
-          <t>-After</t>
+          <t>-BuiltFrom</t>
         </is>
       </c>
       <c r="AJ4" s="25" t="inlineStr">
         <is>
-          <t>-BuiltFrom</t>
+          <t>-FileStem</t>
         </is>
       </c>
       <c r="AK4" s="25" t="inlineStr">
         <is>
-          <t>-FileStem</t>
+          <t>-File</t>
         </is>
       </c>
       <c r="AL4" s="25" t="inlineStr">
         <is>
-          <t>-File</t>
+          <t>-Note</t>
         </is>
       </c>
       <c r="AM4" s="25" t="inlineStr">
         <is>
-          <t>-Note</t>
+          <t>-Against</t>
         </is>
       </c>
       <c r="AN4" s="25" t="inlineStr">
         <is>
-          <t>-Against</t>
+          <t>-Verse</t>
         </is>
       </c>
       <c r="AO4" s="25" t="inlineStr">
         <is>
-          <t>-Verse</t>
+          <t>-Escalation</t>
         </is>
       </c>
       <c r="AP4" s="25" t="inlineStr">
         <is>
-          <t>-Escalation</t>
+          <t>-Thread</t>
         </is>
       </c>
       <c r="AQ4" s="25" t="inlineStr">
         <is>
-          <t>-Thread</t>
+          <t>-NotInNarrative</t>
         </is>
       </c>
       <c r="AR4" s="25" t="inlineStr">
         <is>
-          <t>-NotInNarrative</t>
+          <t>-ToldInMoreThanOne</t>
         </is>
       </c>
       <c r="AS4" s="25" t="inlineStr">
         <is>
-          <t>-ToldInMoreThanOne</t>
-        </is>
-      </c>
-      <c r="AT4" s="25" t="inlineStr">
-        <is>
           <t>-Trace</t>
         </is>
       </c>
+      <c r="AT4" s="25" t="n"/>
     </row>
     <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="C5" t="inlineStr">
         <is>
-          <t>AddClaim|Edit|Tell|Untell|Withdraw|EditNote|EditChapter|EditSection|Record|Find|History|Check|Export</t>
+          <t>AddClaim|Edit|Tell|Untell|Withdraw|EditNote|AddChapter|EditChapter|EditSection|Find|History|Check|Export|QuoteCheck</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5651,107 +5665,137 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>heading text</t>
+          <t>a block: its heading, or 'Parent &gt; Heading' where a heading repeats</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>the passage's opening words</t>
+          <t>in full|in part|pointer</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>in full|in part|pointer</t>
+          <t>which part of the claim the block tells</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>which part of the claim the passage tells</t>
+          <t>EditNote: block heading</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>EditNote: block heading</t>
+          <t>EditNote/EditSection: new heading</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>EditNote/EditSection: new heading</t>
+          <t>order</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>order</t>
+          <t>EditSection: 2-4</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>EditSection: 2-4</t>
+          <t>EditSection: last chapter version</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>EditSection: last chapter version</t>
+          <t>EditChapter: new chapter number</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>EditChapter: new chapter number</t>
+          <t>EditChapter: title</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>EditChapter: title</t>
+          <t>draft|draft + held|empty|deferred</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>draft|draft + held|empty|deferred</t>
+          <t>EditChapter: file name</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>EditChapter: file name</t>
+          <t>EditChapter: version</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>EditChapter: version</t>
+          <t>EditChapter: order in the book</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>EditChapter: order in the book</t>
+          <t>0|1</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>0|1</t>
+          <t>AddChapter/EditChapter: what the chapter is for</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>the ruling, e.g. #2155</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>AddChapter/EditChapter: the chapter before</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>AddChapter</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>AddChapter</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>QuoteCheck: the chapter file</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>Record: the weave update JSON</t>
+          <t>a remark kept on the change rows</t>
         </is>
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>a remark kept on the change rows</t>
+          <t>QuoteCheck: the previous version</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Find: a verse reference</t>
         </is>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>Find: a verse reference</t>
+          <t>Find: escalation id</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>Find: escalation id</t>
+          <t>Find: OT-nn</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>Find: OT-nn</t>
+          <t>Find: switch (x to set)</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
@@ -5760,11 +5804,6 @@
         </is>
       </c>
       <c r="AS5" t="inlineStr">
-        <is>
-          <t>Find: switch (x to set)</t>
-        </is>
-      </c>
-      <c r="AT5" t="inlineStr">
         <is>
           <t>switch (x to set)</t>
         </is>
@@ -5777,7 +5816,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" "&amp;D6&amp;" ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" '"&amp;U6&amp;"' ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6="","",$W$4&amp;" '"&amp;W6&amp;"' ")&amp;IF(X6="","",$X$4&amp;" '"&amp;X6&amp;"' ")&amp;IF(Y6="","",$Y$4&amp;" '"&amp;Y6&amp;"' ")&amp;IF(Z6="","",$Z$4&amp;" '"&amp;Z6&amp;"' ")&amp;IF(AA6="","",$AA$4&amp;" '"&amp;AA6&amp;"' ")&amp;IF(AB6="","",$AB$4&amp;" '"&amp;AB6&amp;"' ")&amp;IF(AC6="","",$AC$4&amp;" '"&amp;AC6&amp;"' ")&amp;IF(AD6="","",$AD$4&amp;" '"&amp;AD6&amp;"' ")&amp;IF(AE6="","",$AE$4&amp;" '"&amp;AE6&amp;"' ")&amp;IF(AF6="","",$AF$4&amp;" '"&amp;AF6&amp;"' ")&amp;IF(AG6="","",$AG$4&amp;" '"&amp;AG6&amp;"' ")&amp;IF(AH6="","",$AH$4&amp;" '"&amp;AH6&amp;"' ")&amp;IF(AI6="","",$AI$4&amp;" '"&amp;AI6&amp;"' ")&amp;IF(AJ6="","",$AJ$4&amp;" '"&amp;AJ6&amp;"' ")&amp;IF(AK6="","",$AK$4&amp;" '"&amp;AK6&amp;"' ")&amp;IF(AL6="","",$AL$4&amp;" '"&amp;AL6&amp;"' ")&amp;IF(AM6="","",$AM$4&amp;" '"&amp;AM6&amp;"' ")&amp;IF(AN6="","",$AN$4&amp;" '"&amp;AN6&amp;"' ")&amp;IF(AO6="","",$AO$4&amp;" '"&amp;AO6&amp;"' ")&amp;IF(AP6="","",$AP$4&amp;" '"&amp;AP6&amp;"' ")&amp;IF(AQ6="","",$AQ$4&amp;" '"&amp;AQ6&amp;"' ")&amp;IF(AR6&lt;&gt;"",$AR$4&amp;" ","")&amp;IF(AS6&lt;&gt;"",$AS$4&amp;" ","")&amp;IF(AT6&lt;&gt;"",$AT$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" "&amp;D6&amp;" ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" '"&amp;U6&amp;"' ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6="","",$W$4&amp;" '"&amp;W6&amp;"' ")&amp;IF(X6="","",$X$4&amp;" '"&amp;X6&amp;"' ")&amp;IF(Y6="","",$Y$4&amp;" '"&amp;Y6&amp;"' ")&amp;IF(Z6="","",$Z$4&amp;" '"&amp;Z6&amp;"' ")&amp;IF(AA6="","",$AA$4&amp;" '"&amp;AA6&amp;"' ")&amp;IF(AB6="","",$AB$4&amp;" '"&amp;AB6&amp;"' ")&amp;IF(AC6="","",$AC$4&amp;" '"&amp;AC6&amp;"' ")&amp;IF(AD6="","",$AD$4&amp;" '"&amp;AD6&amp;"' ")&amp;IF(AE6="","",$AE$4&amp;" '"&amp;AE6&amp;"' ")&amp;IF(AF6="","",$AF$4&amp;" '"&amp;AF6&amp;"' ")&amp;IF(AG6="","",$AG$4&amp;" '"&amp;AG6&amp;"' ")&amp;IF(AH6="","",$AH$4&amp;" '"&amp;AH6&amp;"' ")&amp;IF(AI6="","",$AI$4&amp;" '"&amp;AI6&amp;"' ")&amp;IF(AJ6="","",$AJ$4&amp;" '"&amp;AJ6&amp;"' ")&amp;IF(AK6="","",$AK$4&amp;" '"&amp;AK6&amp;"' ")&amp;IF(AL6="","",$AL$4&amp;" '"&amp;AL6&amp;"' ")&amp;IF(AM6="","",$AM$4&amp;" '"&amp;AM6&amp;"' ")&amp;IF(AN6="","",$AN$4&amp;" '"&amp;AN6&amp;"' ")&amp;IF(AO6="","",$AO$4&amp;" '"&amp;AO6&amp;"' ")&amp;IF(AP6="","",$AP$4&amp;" '"&amp;AP6&amp;"' ")&amp;IF(AQ6&lt;&gt;"",$AQ$4&amp;" ","")&amp;IF(AR6&lt;&gt;"",$AR$4&amp;" ","")&amp;IF(AS6&lt;&gt;"",$AS$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -5795,6 +5834,160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Strand-Reading.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The reading process (escalation #2172): a strand defined, then context, record, gather, map, derive, rewrite and account. Every step dispatches through run.py, work package strand-reading; the JSON shapes are in lib/strandreading.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-Step</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-Strand</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-By</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-Title</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-Cluster</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-Escalation</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-Strongs</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>-Note</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-File</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Define|Context|Record|Gather|Map|Derive|Rewrite|Account</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>the strand's code, e.g. flesh-body</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Claude|Researcher (Define, Context, Record, Map, Derive, Rewrite)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Define: the strand in words</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Define: home cluster, e.g. M48</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Define: the strand's escalation id</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Define: comma-separated exact codes, e.g. H1320,G4561</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Define: a note on the strand or its words</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Record/Map/Derive/Rewrite: the step's JSON</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Strand-Reading.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6&lt;&gt;"",$L$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5871,7 +6064,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5930,108 +6123,6 @@
       </c>
       <c r="B6">
         <f>A6&amp;" "&amp;IF(C6&lt;&gt;"",$C$4&amp;" ","")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>RelationalReading.ps1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>The `verse-reading` stage's RELATIONAL half (`lexical.relational`, escalation #1860 word-level/ relational split, 2026-09-23) -- per-cluster, pre-subgroup Layer 2 pass answering M0.6.5/M0.6.6/ D7.7.1/M0.7.1-16/M0.8.1. Standalone single-step entry point onto the `verse-lexical` work package's `lexical.relational` step (ordinal 7), mirroring `VerseReading.ps1` (`lexical.meaning`, the word-level half) exactly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="25" t="inlineStr">
-        <is>
-          <t>script</t>
-        </is>
-      </c>
-      <c r="B4" s="25" t="inlineStr">
-        <is>
-          <t>compiled command (copy/paste)</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>-ClusterCode</t>
-        </is>
-      </c>
-      <c r="D4" s="25" t="inlineStr">
-        <is>
-          <t>-VerseList</t>
-        </is>
-      </c>
-      <c r="E4" s="25" t="inlineStr">
-        <is>
-          <t>-Live</t>
-        </is>
-      </c>
-      <c r="F4" s="25" t="inlineStr">
-        <is>
-          <t>-Force</t>
-        </is>
-      </c>
-      <c r="G4" s="25" t="inlineStr">
-        <is>
-          <t>-RunId</t>
-        </is>
-      </c>
-      <c r="H4" s="25" t="inlineStr">
-        <is>
-          <t>-Trace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>switch (x to set)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>iba\app\ps\RelationalReading.ps1</t>
-        </is>
-      </c>
-      <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -6112,6 +6203,108 @@
 </file>
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>RelationalReading.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The `verse-reading` stage's RELATIONAL half (`lexical.relational`, escalation #1860 word-level/ relational split, 2026-09-23) -- per-cluster, pre-subgroup Layer 2 pass answering M0.6.5/M0.6.6/ D7.7.1/M0.7.1-16/M0.8.1. Standalone single-step entry point onto the `verse-lexical` work package's `lexical.relational` step (ordinal 7), mirroring `VerseReading.ps1` (`lexical.meaning`, the word-level half) exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>-ClusterCode</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>-VerseList</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>-Live</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>-Force</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>-RunId</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\RelationalReading.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
session 20261023: #2228 the reading process built and closed -- Verse-Scope, Reading-Index, Verse-Collate and Reading.ps1 (three gates: recorded, synergised, published; gap types as config; synergy from the tables); the strand steps retired and the four strands superseded (D-a); analysed set only at gate 1 (D-c); tests 29/29 on a copy (BUILD.md sec 391-398); #2236 Open-Item tool and every open-item thread reworded (295 open, 284 worded; sec 395-397), closed; #2220 SC16 designed stops; #2231-#2234; #2235 held as exception handling; #2237 #2238 raised; the study re-opened (governance.study_status ACTIVE; sec 399)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -53,10 +53,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session-Close" sheetId="45" state="visible" r:id="rId45"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Narrative-Register" sheetId="46" state="visible" r:id="rId46"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strand-Reading" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy-NarrativeToLearning4Comfor" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelationalReading" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run-Stage1Batch" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verse-Scope" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reading-Index" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verse-Collate" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open-Item" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reading" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy-NarrativeToLearning4Comfor" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelationalReading" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run-Stage1Batch" sheetId="56" state="visible" r:id="rId56"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -614,7 +619,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1500,6 +1505,91 @@
         </is>
       </c>
       <c r="C54" t="inlineStr">
+        <is>
+          <t>Retired 2026-10-23 (#2228 D-a): superseded by Reading.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Verse-Scope.ps1</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>The scope resolver (escalation #2228): any request -&gt; the collection of verses as a JSON file under verse_scope.output_dir. Selectors are combined as a union; a bare Strong's code is decomposed to its derivatives; -OnlyStrong narrows the result. Reads only; dispatches through run.py, work package verse-scope.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Reading-Index.ps1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>The cluster reading index (escalation #2228): Build reads the study files under reading_index.roots (only _analytics/Clusters) and records every verse reference with its file, section and line (reading_file, reading_section, reading_ref), incremental and time-guarded; Report writes the coverage report. Dispatches through run.py, work package reading-index.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Verse-Collate.ps1</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>What is known and what is missing for a scope (escalation #2228): the scope resolved as Verse-Scope.ps1 does (same selectors, same guard), then per verse the observations, strand hits, claims, narrative blocks, open items and cluster-file lines, the lexicon per strong, and the gaps; -&gt; verse_collate.output_dir &lt;label&gt;.json and .md. Reads only; dispatches through run.py, work package verse-collate.</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Open-Item.ps1</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Register open items to a clear purpose (escalation #2236): Add, Reword, Split (a target scoped to verses, at most open_item.max_verses; what to read for, why it is open, when it comes back), Due (items that come back when a cluster is worked), Review (stragglers). Dispatches through run.py, work package open-item.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Reading.ps1</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>The reading process (escalation #2228): a reading of one scope through three gates. Open (scope, collation, gap JSON), Record and Check (gate 1: every gap recorded or a reason; verses marked analysed), Synergy, Apply and Check (gate 2: from the tables -- claims, dispositions, tellings, blocks, open items settled), Publish (gate 3: chapters published and copied to learning4comfort), Account. Dispatches through run.py, work package reading.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -5847,11 +5937,10 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The reading process (escalation #2172): a strand defined, then context, record, gather, map, derive, rewrite and account. Every step dispatches through run.py, work package strand-reading; the JSON shapes are in lib/strandreading.py.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>RETIRED 2026-10-23 (#2228 D-a): superseded by Reading.ps1; the script is in iba/app/ps/archive/. The reading process (escalation #2172): a strand defined, then context, record, gather, map, derive, rewrite and account. Every step dispatches through run.py, work package strand-reading; the JSON shapes are in lib/strandreading.py.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -5969,7 +6058,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>iba\app\ps\Strand-Reading.ps1</t>
+          <t>iba\app\ps\archive\Strand-Reading.ps1</t>
         </is>
       </c>
       <c r="B6">
@@ -5988,61 +6077,202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>Compliance.ps1</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Verse-Scope.ps1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The session compliance file (escalation #2173 P2): the governance settings, behaviour rules and escalation rules, restated at start and proved at close.</t>
+          <t>The scope resolver (escalation #2228): any request -&gt; the collection of verses as a JSON file under verse_scope.output_dir. Selectors are combined as a union; a bare Strong's code is decomposed to its derivatives; -OnlyStrong narrows the result. Reads only; dispatches through run.py, work package verse-scope.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>script</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>compiled command (copy/paste)</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>-Action</t>
-        </is>
-      </c>
-      <c r="D4" s="25" t="inlineStr">
-        <is>
-          <t>-Phase</t>
-        </is>
-      </c>
-      <c r="E4" s="25" t="inlineStr">
-        <is>
-          <t>-Mode</t>
-        </is>
-      </c>
-      <c r="F4" s="25" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-Label</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-Cluster</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-Subgroup</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-Strand</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-Word</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-Strong</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-Verse</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>-Chapter</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-Section</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>-Claim</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>-Observation</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-Item</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-Thread</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-File</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-OnlyStrong</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-Reviewed</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>-Trace</t>
         </is>
       </c>
     </row>
     <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>names the output file(s), e.g. anger-bosom</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>e.g. M02 or M02,M01</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>a cluster subgroup code</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>a strand code, e.g. anger</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>a word_registry word</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>e.g. H0430 (bare: all derivatives) or G3563G</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>e.g. Psa 10:2; Luk 14:12-14; Rom 8</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>a narrative chapter, e.g. 10.1</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>with -Chapter: a block heading</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>e.g. C-330</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>an ib_observation id</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>a thread item, e.g. OT-108.3</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>a thread, e.g. OT-108</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>a request JSON file (a batch or kept group)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>filter: keep verses holding one of these codes</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>over 2500 verses: the researcher's review, given after it</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
         <is>
           <t>switch (x to set)</t>
         </is>
@@ -6051,11 +6281,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>iba\app\ps\Compliance.ps1</t>
+          <t>iba\app\ps\Verse-Scope.ps1</t>
         </is>
       </c>
       <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" "&amp;D6&amp;" ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6&lt;&gt;"",$S$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -6070,47 +6300,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>Copy-NarrativeToLearning4Comfort.ps1</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Reading-Index.ps1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Copy the current inner-being narrative files to the learning4comfort publication inbox (escalation #1941). This project never publishes to GitHub itself; the learning4comfort repo prepares, reviews and publishes from its inbox.</t>
+          <t>The cluster reading index (escalation #2228): Build reads the study files under reading_index.roots (only _analytics/Clusters) and records every verse reference with its file, section and line (reading_file, reading_section, reading_ref), incremental and time-guarded; Report writes the coverage report. Dispatches through run.py, work package reading-index.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>script</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>compiled command (copy/paste)</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>-DryRun</t>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-Step</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="C5" t="inlineStr">
         <is>
+          <t>Build|Report</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>switch (x to set)</t>
         </is>
       </c>
@@ -6118,11 +6354,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>iba\app\ps\Copy-NarrativeToLearning4Comfort.ps1</t>
+          <t>iba\app\ps\Reading-Index.ps1</t>
         </is>
       </c>
       <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6&lt;&gt;"",$C$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6&lt;&gt;"",$D$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -6208,6 +6444,864 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:S6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Verse-Collate.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>What is known and what is missing for a scope (escalation #2228): the scope resolved as Verse-Scope.ps1 does (same selectors, same guard), then per verse the observations, strand hits, claims, narrative blocks, open items and cluster-file lines, the lexicon per strong, and the gaps; -&gt; verse_collate.output_dir &lt;label&gt;.json and .md. Reads only; dispatches through run.py, work package verse-collate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-Label</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-Cluster</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-Subgroup</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-Strand</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-Word</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-Strong</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-Verse</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>-Chapter</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-Section</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>-Claim</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>-Observation</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-Item</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-Thread</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-File</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-OnlyStrong</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-Reviewed</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>names the output file(s), e.g. anger-bosom</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>e.g. M02 or M02,M01</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>a cluster subgroup code</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>a strand code, e.g. anger</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>a word_registry word</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>e.g. H0430 (bare: all derivatives) or G3563G</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>e.g. Psa 10:2; Luk 14:12-14; Rom 8</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>a narrative chapter, e.g. 10.1</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>with -Chapter: a block heading</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>e.g. C-330</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>an ib_observation id</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>a thread item, e.g. OT-108.3</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>a thread, e.g. OT-108</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>a request JSON file (a batch or kept group)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>filter: keep verses holding one of these codes</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>over 2500 verses: the researcher's review, given after it</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Verse-Collate.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6&lt;&gt;"",$S$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Open-Item.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Register open items to a clear purpose (escalation #2236): Add, Reword, Split (a target scoped to verses, at most open_item.max_verses; what to read for, why it is open, when it comes back), Due (items that come back when a cluster is worked), Review (stragglers). Dispatches through run.py, work package open-item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-Action</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-Thread</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-Item</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-Origin</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-Anchor</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-Source</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-TargetCluster</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>-TargetTerms</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-Verse</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>-ReadFor</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>-Why</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-ComesBackWhen</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-File</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-Cluster</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-By</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Add|Reword|Split|Due|Review</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Add: OT-nn</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Reword/Split: OT-nn.n</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>the task/issue that raised it</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>strong:|verse:|observation:|claim:|block:</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>the source analysis's strong(s)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>e.g. M58</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>the related term(s) in the target cluster</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>or a verse target</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>what to read for</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>why it is open</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>the trigger</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>a JSON list of specs (Split: the parts)</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Due: the cluster being worked</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Claude|Researcher</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Open-Item.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" "&amp;Q6&amp;" ")&amp;IF(R6&lt;&gt;"",$R$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Reading.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The reading process (escalation #2228): a reading of one scope through three gates. Open (scope, collation, gap JSON), Record and Check (gate 1: every gap recorded or a reason; verses marked analysed), Synergy, Apply and Check (gate 2: from the tables -- claims, dispositions, tellings, blocks, open items settled), Publish (gate 3: chapters published and copied to learning4comfort), Account. Dispatches through run.py, work package reading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-Step</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-Label</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-By</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-Escalation</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-Home</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-Note</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-File</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>-Cluster</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-Subgroup</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>-Strand</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>-Word</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-Strong</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>-Verse</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-Chapter</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-Section</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>-Claim</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>-Observation</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>-Item</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>-Thread</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>-OnlyStrong</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>-Reviewed</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Open|Record|Check|Synergy|Apply|Publish|Account</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>the reading's name</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Claude|Researcher (write steps)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Open: the anchoring task/issue</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Open: the cluster new observations go under</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Open: a note</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Open: a scope request; Record: gap JSON; Apply: synergy JSON</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>scope filter</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>only after the researcher's review (&gt; 2,500 verses)</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Reading.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" '"&amp;U6&amp;"' ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6="","",$W$4&amp;" '"&amp;W6&amp;"' ")&amp;IF(X6&lt;&gt;"",$X$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Compliance.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The session compliance file (escalation #2173 P2): the governance settings, behaviour rules and escalation rules, restated at start and proved at close.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>-Action</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>-Phase</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>-Mode</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Compliance.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" "&amp;D6&amp;" ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Copy-NarrativeToLearning4Comfort.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Copy the current inner-being narrative files to the learning4comfort publication inbox (escalation #1941). This project never publishes to GitHub itself; the learning4comfort repo prepares, reviews and publishes from its inbox.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>-DryRun</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Copy-NarrativeToLearning4Comfort.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6&lt;&gt;"",$C$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6304,7 +7398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
session 20261023: #2212 the prose patch apply back as a registered step -- prose.apply_patch (Prose.ps1 -Step ApplyPatch -PatchFile [-DryRun], iba/app/lib/prosestore.py apply_patch / run_apply_patch), the prose operations of the archived apply_session_patch.py in one transaction through the record_change_log choke point, writing only the tables granted to writer apply_session_patch; option A chosen and approved by the researcher, built in standard mode with #2241-#2243 applied through configmaint.propose; tests 11/11 on database copies plus 8a and 8b live (BUILD.md sec 400); #2166 closed by the researcher; #2244 test artefact resolved; #2245 raised (SC16 and test refusals)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -2707,7 +2707,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2725,7 +2725,7 @@
     <row r="2" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Prose store: extract/search/export/import/flag/status the programme prose.</t>
+          <t>Prose store: extract/search/export/import/flag/status the programme prose, and apply the reviewed patch.</t>
         </is>
       </c>
     </row>
@@ -2838,10 +2838,20 @@
       </c>
       <c r="V4" s="4" t="inlineStr">
         <is>
+          <t>-PatchFile</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>-DryRun</t>
+        </is>
+      </c>
+      <c r="X4" s="4" t="inlineStr">
+        <is>
           <t>-Out</t>
         </is>
       </c>
-      <c r="W4" s="4" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>-Trace</t>
         </is>
@@ -2850,7 +2860,7 @@
     <row r="5" ht="18.75" customFormat="1" customHeight="1" s="18">
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>Extract|Search|ExportChapter|ImportChapter|Flag|FlagFixPropose|FlagFixApply|SetStatus</t>
+          <t>Extract|Search|ExportChapter|ImportChapter|Flag|FlagFixPropose|FlagFixApply|SetStatus|ApplyPatch</t>
         </is>
       </c>
       <c r="D5" s="17" t="inlineStr">
@@ -2909,6 +2919,16 @@
         </is>
       </c>
       <c r="V5" s="17" t="inlineStr">
+        <is>
+          <t>ApplyPatch: patch .json</t>
+        </is>
+      </c>
+      <c r="W5" s="17" t="inlineStr">
+        <is>
+          <t>ApplyPatch: roll back</t>
+        </is>
+      </c>
+      <c r="X5" s="17" t="inlineStr">
         <is>
           <t>override output path</t>
         </is>
@@ -2921,7 +2941,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6="","",$F$4&amp;" "&amp;F6&amp;" ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")&amp;IF(I6&lt;&gt;"",$I$4&amp;" ","")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" "&amp;K6&amp;" ")&amp;IF(L6&lt;&gt;"",$L$4&amp;" ","")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" "&amp;U6&amp;" ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6&lt;&gt;"",$W$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6="","",$F$4&amp;" "&amp;F6&amp;" ")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")&amp;IF(H6&lt;&gt;"",$H$4&amp;" ","")&amp;IF(I6&lt;&gt;"",$I$4&amp;" ","")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" "&amp;K6&amp;" ")&amp;IF(L6&lt;&gt;"",$L$4&amp;" ","")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" "&amp;U6&amp;" ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6&lt;&gt;"",$W$4&amp;" ","")&amp;IF(X6="","",$X$4&amp;" '"&amp;X6&amp;"' ")&amp;IF(Y6&lt;&gt;"",$Y$4&amp;" ","")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
session 20261024: #2273 and #2274 (#2268 B1, B2) the reading on its phases and the observation record as findings and their nodes; design v1 to v6 on the researcher's corrections (the observation/node model inspected, parties as findings, ledgers and catalogue compared, qualifiers read for value); built as one change set (159 config writes, observationrecord.py, Reading.ps1 Gather/Observe/Narrate and four gates), tested 47/47 on a copy, applied live, accepted (BUILD.md 408)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -6900,7 +6900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6913,7 +6913,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The reading process (escalation #2228): a reading of one scope through three gates. Open (scope, collation, gap JSON), Record and Check (gate 1: every gap recorded or a reason; verses marked analysed), Synergy, Apply and Check (gate 2: from the tables -- claims, dispositions, tellings, blocks, open items settled), Publish (gate 3: chapters published and copied to learning4comfort), Account. Dispatches through run.py, work package reading.</t>
+          <t>The reading process (escalations #2228, #2273): a reading of one scope with its objective, on the phases, through four gates. Open (0.C: scope, objective, collation, pre-gap JSON), Gather and Check (pre gate), Observe, Record and Check (observe gate: every word in focus, qualifiers included, has a finding of this reading, an open item or a reason; verses marked analysed), Synergy, Apply and Check (claims gate: every node disposed, every claim on a finding), Narrate and Check (narrate gate: every claim told or held), Publish, Account. Findings: one observation each, applied by nodes. Dispatches through run.py, work package reading.</t>
         </is>
       </c>
     </row>
@@ -6955,85 +6955,90 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>-Objective</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>-Note</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>-File</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>-Cluster</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>-Subgroup</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>-Strand</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>-Word</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>-Strong</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>-Verse</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>-Chapter</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>-Section</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>-Claim</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>-Observation</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>-Item</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>-Thread</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>-OnlyStrong</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>-Reviewed</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>-Trace</t>
         </is>
@@ -7042,7 +7047,7 @@
     <row r="5">
       <c r="C5" t="inlineStr">
         <is>
-          <t>Open|Record|Check|Synergy|Apply|Publish|Account</t>
+          <t>Open|Gather|Observe|Record|Check|Synergy|Apply|Narrate|Publish|Account</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -7062,90 +7067,95 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Open: the cluster new observations go under</t>
+          <t>Open: the cluster the scope is anchored on (alias -Home)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>Open: the scope's objective (0.C), in words</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>Open: a note</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Open: a scope request; Record: gap JSON; Apply: synergy JSON</t>
-        </is>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>Open: a scope request; Gather: pre-gap JSON; Record: observe JSON; Apply: synergy JSON; Narrate: narrate JSON</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>scope filter</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>only after the researcher's review (&gt; 2,500 verses)</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>switch (x to set)</t>
         </is>
@@ -7158,7 +7168,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" '"&amp;U6&amp;"' ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6="","",$W$4&amp;" '"&amp;W6&amp;"' ")&amp;IF(X6&lt;&gt;"",$X$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" '"&amp;U6&amp;"' ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6="","",$W$4&amp;" '"&amp;W6&amp;"' ")&amp;IF(X6="","",$X$4&amp;" '"&amp;X6&amp;"' ")&amp;IF(Y6&lt;&gt;"",$Y$4&amp;" ","")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
session 20261026: #2286 U1 to U4 and U8 built in Developer Mode: surface subgroup rules (#2291), schema (#2292), the cluster.surface_map steps and Surface-Map.ps1 (#2293), the reading gate (#2294); pilot on M18 and M67 and the bulk mapping of all 80 M clusters (#2298, 13,411 pairs); Q1 to Q4 answered, RO13 segment-large-subgroup into config; #2300 self-corrected; #2301 backup taken, pruning held to 2026-10-28
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -62,6 +62,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Copy-NarrativeToLearning4Comfor" sheetId="54" state="visible" r:id="rId54"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelationalReading" sheetId="55" state="visible" r:id="rId55"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run-Stage1Batch" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Surface-Map" sheetId="57" state="visible" r:id="rId57"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -619,7 +620,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1590,6 +1591,23 @@
         </is>
       </c>
       <c r="C59" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Surface-Map.ps1</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>The surface mapping of an M cluster (escalation #2293, #2286 U3): Pairs writes the pairs file; Claude fills the groups and head; Apply writes it; Tail places the rest by the API (a preview unless -Live); Check reports group sizes, anomalies, unallocated and two-sense pairs. Dispatches through run.py, work package cluster-surface-map.</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -7520,6 +7538,110 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Surface-Map.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The surface mapping of an M cluster (escalation #2293, #2286 U3): Pairs writes the pairs file; Claude fills the groups and head; Apply writes it; Tail places the rest by the API (a preview unless -Live); Check reports group sizes, anomalies, unallocated and two-sense pairs. Dispatches through run.py, work package cluster-surface-map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-Step</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-Cluster</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-File</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-Live</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Pairs | Apply | Tail | Check</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>an M cluster, e.g. M18</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>with Apply: the filled pairs file</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>with Tail: switch (x to set): call the API; without it a preview</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Surface-Map.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
session 20261026: #2286 finished and closed: U5 occurrence-shaped scope resolver (#2295, with #2287), U7 method rule RA-01 (#2297), U9 cluster.subgroup pipeline retired in config (#2299), U6 on hold (#2296); #2303 raised; #2304 reading cycle on one JSON designed (v3) and prototyped on M18_thirst on a copy, then parked; #2305 raised to capture prior reading work into ib_observation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -6115,8 +6115,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6128,10 +6132,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The scope resolver (escalation #2228): any request -&gt; the collection of verses as a JSON file under verse_scope.output_dir. Selectors are combined as a union; a bare Strong's code is decomposed to its derivatives; -OnlyStrong narrows the result. Reads only; dispatches through run.py, work package verse-scope.</t>
-        </is>
-      </c>
-    </row>
+          <t>The scope resolver (escalations #2228, #2295): any request -&gt; the collection of verses with their occurrences as a JSON file under verse_scope.output_dir. Selectors are combined as a union; a bare Strong's code is decomposed to its derivatives; a mapped M cluster or a subgroup enters through its (code, surface) pairs, a word through its surface; -HomeScope (alias -Home) names the home; -OnlyStrong narrows the result. Reads only; dispatches through run.py, work package verse-scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -6208,22 +6213,27 @@
           <t>-Thread</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" s="23" t="inlineStr">
+        <is>
+          <t>-HomeScope</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>-File</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>-OnlyStrong</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>-Reviewed</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>-Trace</t>
         </is>
@@ -6295,22 +6305,27 @@
           <t>a thread, e.g. OT-108</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P5" s="23" t="inlineStr">
+        <is>
+          <t>the home: a subgroup or an M cluster (alias -Home), when not the ones named</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>a request JSON file (a batch or kept group)</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>filter: keep verses holding one of these codes</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>over 2500 verses: the researcher's review, given after it</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>switch (x to set)</t>
         </is>
@@ -6323,7 +6338,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6&lt;&gt;"",$S$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6&lt;&gt;"",$T$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -7544,7 +7559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7561,7 +7576,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
session 20261026: #2305 prior-work capture built, piloted and applied live: Prior-Capture.ps1 (Prepare, Record, Report), table prior_capture_line, stage prior-capture, tag unfitted, method rules CP-01 to CP-10 (D1 to D3 ruled), migration 63 writes, 48 of 48 tests; run live on M01, M02, M07, M08 and M09: 62 of 235 documents, 3,146 observations; #2306 and #2302 resolved; session log and compliance file
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -63,6 +63,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelationalReading" sheetId="55" state="visible" r:id="rId55"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run-Stage1Batch" sheetId="56" state="visible" r:id="rId56"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Surface-Map" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prior-Capture" sheetId="58" state="visible" r:id="rId58"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -620,7 +621,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1608,6 +1609,23 @@
         </is>
       </c>
       <c r="C60" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Prior-Capture.ps1</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>The capture of prior study documents into the observation record (escalation #2305): Prepare writes the document's JSON (lines that name a verse, verses resolved, M/T-coded words, October ids); Claude fills findings and an answer per line; Record writes it whole or refuses it whole; Report shows where the capture stands. Dispatches through run.py, work package prior-capture.</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -6136,7 +6154,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -7648,6 +7665,89 @@
       </c>
       <c r="B6">
         <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" '"&amp;E6&amp;"' ")&amp;IF(F6&lt;&gt;"",$F$4&amp;" ","")&amp;IF(G6&lt;&gt;"",$G$4&amp;" ","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Prior-Capture.ps1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The capture of prior study documents into the observation record (escalation #2305): Prepare writes the document's JSON (lines that name a verse, verses resolved, M/T-coded words, October ids); Claude fills findings and an answer per line; Record writes it whole or refuses it whole; Report shows where the capture stands. Dispatches through run.py, work package prior-capture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>script</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>compiled command (copy/paste)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-Step</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-File</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-Trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Prepare | Record | Report</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>with Prepare: the document's repo-relative path or reading_file id; with Record: the filled JSON</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>switch (x to set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>iba\app\ps\Prior-Capture.ps1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" '"&amp;C6&amp;"' ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6&lt;&gt;"",$E$4&amp;" ","")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
session 20261027: Analysis_phase_1 specification v4 (#2318, #2319) and the build to it (#2320): scope JSON as index, query by verse, accept/modify/soft delete, new gate; migrations, tests, docs; session log and close reports
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/ps tools worksheet.xlsx
+++ b/iba/docs/ps tools worksheet.xlsx
@@ -6950,8 +6950,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y6"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6963,7 +6968,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The reading process (escalations #2228, #2273): a reading of one scope with its objective, on the phases, through four gates. Open (0.C: scope, objective, collation, pre-gap JSON), Gather and Check (pre gate), Observe, Record and Check (observe gate: every word in focus, qualifiers included, has a finding of this reading, an open item or a reason; verses marked analysed), Synergy, Apply and Check (claims gate: every node disposed, every claim on a finding), Narrate and Check (narrate gate: every claim told or held), Publish, Account. Findings: one observation each, applied by nodes. Dispatches through run.py, work package reading.</t>
+          <t>The reading process (escalations #2228, #2273, #2320). Analysis_phase_1 (the verse understanding): Open (0.C: ONE subgroup or a segment of it; the scope JSON that indexes the verses), Observe (the next verses in hand: each verse's sheet is read from the tables now), Record (the filled sheets: each surface evaluated, each existing observation and node accepted, modified or soft deleted, new findings written), Check (the Observe gate: every verse done; verses marked analysed). Gather is retired. Then Synergy, Apply and Check (claims gate), Narrate and Check (narrate gate), Publish, Account. Dispatches through run.py, work package reading.</t>
         </is>
       </c>
     </row>
@@ -7093,11 +7098,21 @@
           <t>-Trace</t>
         </is>
       </c>
+      <c r="Z4" s="23" t="inlineStr">
+        <is>
+          <t>-Surface</t>
+        </is>
+      </c>
+      <c r="AA4" s="23" t="inlineStr">
+        <is>
+          <t>-Count</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="C5" t="inlineStr">
         <is>
-          <t>Open|Gather|Observe|Record|Check|Synergy|Apply|Narrate|Publish|Account</t>
+          <t>Open|Observe|Record|Check|Synergy|Apply|Narrate|Publish|Account</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -7117,7 +7132,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Open: the cluster the scope is anchored on (alias -Home)</t>
+          <t>not given for Open: the home is the subgroup's cluster (alias -Home)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -7132,69 +7147,69 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Open: a scope request; Gather: pre-gap JSON; Record: observe JSON; Apply: synergy JSON; Narrate: narrate JSON</t>
+          <t>Apply: synergy JSON; Narrate: narrate JSON (Open takes no request file)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>not for Analysis_phase_1</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Open: the ONE subgroup, which is the home</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Open: a segment (verses of the subgroup); Observe: the verse to put in hand</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>scope</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>scope</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>scope</t>
-        </is>
-      </c>
       <c r="W5" t="inlineStr">
         <is>
           <t>scope filter</t>
@@ -7208,6 +7223,16 @@
       <c r="Y5" t="inlineStr">
         <is>
           <t>switch (x to set)</t>
+        </is>
+      </c>
+      <c r="Z5" s="23" t="inlineStr">
+        <is>
+          <t>Open: a segment (surfaces of the subgroup, comma list)</t>
+        </is>
+      </c>
+      <c r="AA5" s="23" t="inlineStr">
+        <is>
+          <t>Observe: how many verses to put in hand (default reading.verse_loop)</t>
         </is>
       </c>
     </row>
@@ -7218,7 +7243,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" '"&amp;U6&amp;"' ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6="","",$W$4&amp;" '"&amp;W6&amp;"' ")&amp;IF(X6="","",$X$4&amp;" '"&amp;X6&amp;"' ")&amp;IF(Y6&lt;&gt;"",$Y$4&amp;" ","")</f>
+        <f>A6&amp;" "&amp;IF(C6="","",$C$4&amp;" "&amp;C6&amp;" ")&amp;IF(D6="","",$D$4&amp;" '"&amp;D6&amp;"' ")&amp;IF(E6="","",$E$4&amp;" "&amp;E6&amp;" ")&amp;IF(F6="","",$F$4&amp;" '"&amp;F6&amp;"' ")&amp;IF(G6="","",$G$4&amp;" '"&amp;G6&amp;"' ")&amp;IF(H6="","",$H$4&amp;" '"&amp;H6&amp;"' ")&amp;IF(I6="","",$I$4&amp;" '"&amp;I6&amp;"' ")&amp;IF(J6="","",$J$4&amp;" '"&amp;J6&amp;"' ")&amp;IF(K6="","",$K$4&amp;" '"&amp;K6&amp;"' ")&amp;IF(L6="","",$L$4&amp;" '"&amp;L6&amp;"' ")&amp;IF(M6="","",$M$4&amp;" '"&amp;M6&amp;"' ")&amp;IF(N6="","",$N$4&amp;" '"&amp;N6&amp;"' ")&amp;IF(O6="","",$O$4&amp;" '"&amp;O6&amp;"' ")&amp;IF(P6="","",$P$4&amp;" '"&amp;P6&amp;"' ")&amp;IF(Q6="","",$Q$4&amp;" '"&amp;Q6&amp;"' ")&amp;IF(R6="","",$R$4&amp;" '"&amp;R6&amp;"' ")&amp;IF(S6="","",$S$4&amp;" '"&amp;S6&amp;"' ")&amp;IF(T6="","",$T$4&amp;" '"&amp;T6&amp;"' ")&amp;IF(U6="","",$U$4&amp;" '"&amp;U6&amp;"' ")&amp;IF(V6="","",$V$4&amp;" '"&amp;V6&amp;"' ")&amp;IF(W6="","",$W$4&amp;" '"&amp;W6&amp;"' ")&amp;IF(X6="","",$X$4&amp;" '"&amp;X6&amp;"' ")&amp;IF(Z6="","",$Z$4&amp;" '"&amp;Z6&amp;"' ")&amp;IF(AA6="","",$AA$4&amp;" '"&amp;AA6&amp;"' ")&amp;IF(Y6&lt;&gt;"",$Y$4&amp;" ","")</f>
         <v/>
       </c>
     </row>
@@ -7679,7 +7704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">

</xml_diff>